<commit_message>
feat: 战斗对象通用预制体(common_battle嵌套) + npc/talk目录拆分 + 修复Spine材质引用/meta冲突 + 删冗余PlayerCharacter2D
</commit_message>
<xml_diff>
--- a/DataTables/Datas/person.xlsx
+++ b/DataTables/Datas/person.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="person" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="person" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="P5" s="1" t="inlineStr">
         <is>
-          <t>prefabs/npc/coach</t>
+          <t>prefabs/npc/talk/coach</t>
         </is>
       </c>
       <c r="Q5" s="1" t="inlineStr">

</xml_diff>